<commit_message>
Feat T029-T034: Validação da importação com dados anonimizados
</commit_message>
<xml_diff>
--- a/data/legado-solides/samples/avaliacoes_crosswalk_min.xlsx
+++ b/data/legado-solides/samples/avaliacoes_crosswalk_min.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Avaliacoes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,77 +427,111 @@
           <t>Identificador Avaliado</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Identificador</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Identificador Solicitação</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ana Silva</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>101</t>
-        </is>
+          <t>Gestor Alpha</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>100</v>
+      </c>
+      <c r="C2" t="n">
+        <v>5100</v>
+      </c>
+      <c r="D2" t="n">
+        <v>8001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Bruno Costa</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>102</t>
-        </is>
+          <t>Ana Silva</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>101</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5101</v>
+      </c>
+      <c r="D3" t="n">
+        <v>8001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Carla Dias</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>103</t>
-        </is>
+          <t>Bruno Costa</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>102</v>
+      </c>
+      <c r="C4" t="n">
+        <v>5102</v>
+      </c>
+      <c r="D4" t="n">
+        <v>8001</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Diego Alves</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>104</t>
-        </is>
+          <t>Carla Dias</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>103</v>
+      </c>
+      <c r="C5" t="n">
+        <v>5103</v>
+      </c>
+      <c r="D5" t="n">
+        <v>8001</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Fernanda Lima</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>105</t>
-        </is>
+          <t>Diego Alves</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>104</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5104</v>
+      </c>
+      <c r="D6" t="n">
+        <v>8001</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Gestor Alpha</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
+          <t>Nome Ambiguo</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>900</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5900</v>
+      </c>
+      <c r="D7" t="n">
+        <v>8001</v>
       </c>
     </row>
     <row r="8">
@@ -506,22 +540,14 @@
           <t>Nome Ambiguo</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>900</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Nome Ambiguo</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>901</t>
-        </is>
+      <c r="B8" t="n">
+        <v>901</v>
+      </c>
+      <c r="C8" t="n">
+        <v>5901</v>
+      </c>
+      <c r="D8" t="n">
+        <v>8001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>